<commit_message>
Corrige el corte: dos entregas que estaban en ramas viejas y no se habian visto
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S02-corte-07sep.xlsx
+++ b/calificaciones/P00-S02-corte-07sep.xlsx
@@ -12,18 +12,16 @@
     <sheet name="321132477" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="320298835" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="117003136" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="321058526" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="320152841" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="318586465" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="320018277" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="320229594" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="320250648" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="319659852" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="320187072" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="320229264" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="320284858" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="320224159" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="320049376" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="320152841" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="318586465" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="320018277" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="320229594" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="320250648" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="319659852" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="320229264" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="320284858" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="320224159" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="320049376" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1068,14 +1066,14 @@
           <t>321058526</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
@@ -1095,7 +1093,7 @@
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>Tu S02 solo tiene un hola_mundo.py: faltan el Dockerfile, la evidencia y el index.html. Y falta tu p00.</t>
+          <t>Completa. Tu entrega estaba en tu rama vieja y no la habiamos visto: ya la consolidamos en tu rama. Tu evidencia esta muy bien. Detalle menor: en p00 te quedaron archivos de mas.</t>
         </is>
       </c>
     </row>
@@ -1813,9 +1811,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>parcial</t>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
@@ -1835,7 +1833,7 @@
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>Te falto contestar la segunda pregunta. Ver tu hoja.</t>
+          <t>Completa y correcta.</t>
         </is>
       </c>
     </row>
@@ -2256,14 +2254,14 @@
     <row r="52">
       <c r="A52" s="13" t="inlineStr">
         <is>
-          <t>P00 entregada: 37 / 43   (de esas, 4 sin el nombre adentro)</t>
+          <t>P00 entregada: 38 / 43   (de esas, 4 sin el nombre adentro)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="13" t="inlineStr">
         <is>
-          <t>S02 completa: 30 / 43   ·   parcial: 8   ·   sin entregar: 5</t>
+          <t>S02 completa: 32 / 43   ·   parcial: 7   ·   sin entregar: 4</t>
         </is>
       </c>
     </row>
@@ -2309,14 +2307,14 @@
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Correccion · 320229594</t>
+          <t>Correccion · 320250648</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320229594   ·   Por corregir: S02 y p00</t>
+          <t>Cuenta: 320250648   ·   Por corregir: p00</t>
         </is>
       </c>
     </row>
@@ -2342,7 +2340,7 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Tu p00 no lleva tu nombre: dice 'Esta es una prueba de git'.</t>
+          <t>Tu p00 no lleva tu nombre.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
@@ -2354,12 +2352,12 @@
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Escribes docker build -t mi-sitio-v2 sin el punto final, y usas mi-sitio-v2 como si fuera la version 2.</t>
+          <t>Tu carpeta se llama Salgado_Roman con mayusculas.</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>El punto es obligatorio: dice donde esta el Dockerfile. Y la version 2 se marca con dos puntos: mi-sitio:v2, no con guion.</t>
+          <t>Deberia ir en minusculas: apellido_nombre.</t>
         </is>
       </c>
     </row>
@@ -2430,7 +2428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -2440,21 +2438,21 @@
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Correccion · 320250648</t>
+          <t>Correccion · 319659852</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320250648   ·   Por corregir: p00</t>
+          <t>Cuenta: 319659852   ·   Por corregir: S02 y p00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: sin nombre      S02: ✓      L2: ✓</t>
+          <t>P00: ✗      S02: parcial      L2: ✗</t>
         </is>
       </c>
     </row>
@@ -2473,78 +2471,90 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Tu p00 no lleva tu nombre.</t>
+          <t>Falta el error de puerto ocupado: no aparece en tu evidencia.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Abrelo, escribe tu nombre completo y haz push.</t>
+          <t>Levanta dos contenedores en el mismo puerto; el segundo falla con 'port is already allocated'. Pega ese texto.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Tu carpeta se llama Salgado_Roman con mayusculas.</t>
+          <t>No tienes p00.</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Deberia ir en minusculas: apellido_nombre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+          <t>Crea entregas/tu_carpeta/p00/prueba.txt con tu nombre completo y haz push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Tu Dockerfile es el unico sin EXPOSE 80.</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Construye igual, pero agregalo: documenta que el contenedor escucha en el 80.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>git commit -m "S02: correccion"</t>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="18" t="inlineStr">
         <is>
+          <t>git commit -m "S02: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
           <t>git push</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2571,21 +2581,21 @@
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Correccion · 319659852</t>
+          <t>Correccion · 320229264</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 319659852   ·   Por corregir: S02 y p00</t>
+          <t>Cuenta: 320229264   ·   Por corregir: S02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: ✗      S02: parcial      L2: ✗</t>
+          <t>P00: ✓      S02: parcial      L2: ✗</t>
         </is>
       </c>
     </row>
@@ -2604,36 +2614,36 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Falta el error de puerto ocupado: no aparece en tu evidencia.</t>
+          <t>El docker ps que pegaste no muestra tus contenedores: salen miweb, web1 y web2, no los tuyos. La mision 3 se queda sin evidencia.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Levanta dos contenedores en el mismo puerto; el segundo falla con 'port is already allocated'. Pega ese texto.</t>
+          <t>Levanta TUS dos contenedores con --name sitio y --name sitio2, corre docker ps y pega esa salida.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>No tienes p00.</t>
+          <t>El error de puerto lo describes con tus palabras ('Docker mostro un error equivalente al siguiente') en vez de pegarlo.</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Crea entregas/tu_carpeta/p00/prueba.txt con tu nombre completo y haz push.</t>
+          <t>Reproducelo y pega el texto tal cual sale en tu terminal.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>Tu Dockerfile es el unico sin EXPOSE 80.</t>
+          <t>Tu index.html no trae la tabla de 5 comandos.</t>
         </is>
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>Construye igual, pero agregalo: documenta que el contenedor escucha en el 80.</t>
+          <t>Esa era la mision 1: agregala.</t>
         </is>
       </c>
     </row>
@@ -2714,21 +2724,21 @@
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Correccion · 320187072</t>
+          <t>Correccion · 320284858</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320187072   ·   Por corregir: S02</t>
+          <t>Cuenta: 320284858   ·   Por corregir: p00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: parcial      L2: ✓</t>
+          <t>P00: sin nombre      S02: ✓      L2: ✗</t>
         </is>
       </c>
     </row>
@@ -2747,12 +2757,12 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Solo contestaste la primera pregunta. Falta: que comparten y que no comparten dos contenedores de la misma imagen.</t>
+          <t>Tu p00 dice solo 'prueba', sin tu nombre.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Contestala en tu evidencia.md. Pista: comparten la imagen (las capas de solo lectura); no comparten su capa de escritura ni su puerto en el host.</t>
+          <t>Abrelo, escribe tu nombre completo y haz push. Tu S02 esta completa.</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -2833,21 +2843,21 @@
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Correccion · 320229264</t>
+          <t>Correccion · 320224159</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320229264   ·   Por corregir: S02</t>
+          <t>Cuenta: 320224159   ·   Por corregir: S02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: parcial      L2: ✗</t>
+          <t>P00: ✓      S02: parcial      L2: ✓</t>
         </is>
       </c>
     </row>
@@ -2866,90 +2876,66 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>El docker ps que pegaste no muestra tus contenedores: salen miweb, web1 y web2, no los tuyos. La mision 3 se queda sin evidencia.</t>
+          <t>Tu evidencia.md esta cortada a la mitad: son 516 caracteres y termina a media instruccion, despues de la lista de comandos.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Levanta TUS dos contenedores con --name sitio y --name sitio2, corre docker ps y pega esa salida.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>El error de puerto lo describes con tus palabras ('Docker mostro un error equivalente al siguiente') en vez de pegarlo.</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>Reproducelo y pega el texto tal cual sale en tu terminal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>Tu index.html no trae la tabla de 5 comandos.</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>Esa era la mision 1: agregala.</t>
+          <t>Falta el docker ps, el error de puerto ocupado y las dos respuestas. Probablemente no guardaste antes de subir: completala y vuelve a hacer push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t>git checkout TU-RAMA</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="18" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
+          <t>git push</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2976,244 +2962,6 @@
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Correccion · 320284858</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 320284858   ·   Por corregir: p00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>P00: sin nombre      S02: ✓      L2: ✗</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>Tu p00 dice solo 'prueba', sin tu nombre.</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Abrelo, escribe tu nombre completo y haz push. Tu S02 esta completa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="17" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="14" t="inlineStr">
-        <is>
-          <t>Correccion · 320224159</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 320224159   ·   Por corregir: S02</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>P00: ✓      S02: parcial      L2: ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>Tu evidencia.md esta cortada a la mitad: son 516 caracteres y termina a media instruccion, despues de la lista de comandos.</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Falta el docker ps, el error de puerto ocupado y las dos respuestas. Probablemente no guardaste antes de subir: completala y vuelve a hacer push.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="17" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="14" t="inlineStr">
-        <is>
           <t>Correccion · 320049376</t>
         </is>
       </c>
@@ -3845,21 +3593,21 @@
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Correccion · 321058526</t>
+          <t>Correccion · 320152841</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 321058526   ·   Por corregir: S02 y p00</t>
+          <t>Cuenta: 320152841   ·   Por corregir: S02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: ✗      S02: ✗      L2: ✓</t>
+          <t>P00: ✓      S02: ✓      L2: ✗</t>
         </is>
       </c>
     </row>
@@ -3878,24 +3626,24 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Tu s02 solo tiene un hola_mundo.py. Falta el Dockerfile, el index.html y la evidencia.md: practicamente todo el laboratorio.</t>
+          <t>Tu respuesta de por que la pagina no cambio esta equivocada: dices que Docker bloquea la imagen.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Sigue la guia en labs/Lab-S02-Docker-dia-1.html desde el principio y sube los tres archivos.</t>
+          <t>La razon es que la imagen es inmutable: el contenedor sigue corriendo la imagen vieja, y hasta que no reconstruyes con docker build no existe una imagen nueva.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>No tienes p00, que era la tarea de Git.</t>
+          <t>Tu carpeta lleva solo tu apellido.</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Crea entregas/tu_carpeta/p00/prueba.txt con tu nombre completo adentro y haz push.</t>
+          <t>Deberia ser apellido_nombre, igual que tu rama.</t>
         </is>
       </c>
     </row>
@@ -3976,21 +3724,21 @@
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Correccion · 320152841</t>
+          <t>Correccion · 318586465</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320152841   ·   Por corregir: S02</t>
+          <t>Cuenta: 318586465   ·   Por corregir: S02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: ✓      L2: ✗</t>
+          <t>P00: ✓      S02: parcial      L2: ✓</t>
         </is>
       </c>
     </row>
@@ -4009,24 +3757,24 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Tu respuesta de por que la pagina no cambio esta equivocada: dices que Docker bloquea la imagen.</t>
+          <t>Falta la salida de docker ps (mision 3): no aparece en tu evidencia.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>La razon es que la imagen es inmutable: el contenedor sigue corriendo la imagen vieja, y hasta que no reconstruyes con docker build no existe una imagen nueva.</t>
+          <t>Con tus dos contenedores corriendo, ejecuta docker ps y pega la salida COMPLETA en tu evidencia.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Tu carpeta lleva solo tu apellido.</t>
+          <t>Tu archivo se llama evindecia.md.</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Deberia ser apellido_nombre, igual que tu rama.</t>
+          <t>Renombralo a evidencia.md.</t>
         </is>
       </c>
     </row>
@@ -4092,6 +3840,125 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Correccion · 320018277</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 320018277   ·   Por corregir: S02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>P00: ✓      S02: parcial      L2: ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="56" customHeight="1">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Tu evidencia trae el texto de ejemplo de la guia sin llenar: bajo Mision 3 dice literalmente '[Aqui va el texto que te salio cuando hiciste docker ps]'. Nunca pegaste tu salida real.</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>Corre docker ps con tus contenedores arriba y sustituye ese renglon por lo que te salga. Lo que se califica es tu evidencia, no la plantilla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>git commit -m "S02: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4107,21 +3974,21 @@
     <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>Correccion · 318586465</t>
+          <t>Correccion · 320229594</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 318586465   ·   Por corregir: S02</t>
+          <t>Cuenta: 320229594   ·   Por corregir: S02 y p00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: parcial      L2: ✓</t>
+          <t>P00: sin nombre      S02: ✓      L2: ✓</t>
         </is>
       </c>
     </row>
@@ -4140,24 +4007,24 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>Falta la salida de docker ps (mision 3): no aparece en tu evidencia.</t>
+          <t>Tu p00 no lleva tu nombre: dice 'Esta es una prueba de git'.</t>
         </is>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Con tus dos contenedores corriendo, ejecuta docker ps y pega la salida COMPLETA en tu evidencia.</t>
+          <t>Abrelo, escribe tu nombre completo y haz push.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Tu archivo se llama evindecia.md.</t>
+          <t>Escribes docker build -t mi-sitio-v2 sin el punto final, y usas mi-sitio-v2 como si fuera la version 2.</t>
         </is>
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>Renombralo a evidencia.md.</t>
+          <t>El punto es obligatorio: dice donde esta el Dockerfile. Y la version 2 se marca con dos puntos: mi-sitio:v2, no con guion.</t>
         </is>
       </c>
     </row>
@@ -4212,125 +4079,6 @@
     </row>
     <row r="16">
       <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="14" t="inlineStr">
-        <is>
-          <t>Correccion · 320018277</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 320018277   ·   Por corregir: S02</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>P00: ✓      S02: parcial      L2: ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="56" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>Tu evidencia trae el texto de ejemplo de la guia sin llenar: bajo Mision 3 dice literalmente '[Aqui va el texto que te salio cuando hiciste docker ps]'. Nunca pegaste tu salida real.</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Corre docker ps con tus contenedores arriba y sustituye ese renglon por lo que te salga. Lo que se califica es tu evidencia, no la plantilla.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="17" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="18" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>

</xml_diff>

<commit_message>
Corrige la atribucion de dos usuarios de GitHub en el registro de lecturas
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S02-corte-07sep.xlsx
+++ b/calificaciones/P00-S02-corte-07sep.xlsx
@@ -780,14 +780,14 @@
           <t>✗</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>tarde</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>Falta toda la S02.</t>
+          <t>Tus lecturas SI estan registradas. Falta la S02: cuando la subas se actualiza.</t>
         </is>
       </c>
     </row>
@@ -2223,14 +2223,14 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D49" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>tarde</t>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F49" s="9" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="G49" s="10" t="inlineStr">
         <is>
-          <t>Tu S02 esta completa, pero falta tu p00.</t>
+          <t>Tu S02 esta completa y tu lectura entro en tiempo. Falta tu p00.</t>
         </is>
       </c>
     </row>
@@ -2268,7 +2268,7 @@
     <row r="54">
       <c r="A54" s="13" t="inlineStr">
         <is>
-          <t>Lectura 2: 30 en tiempo + 5 tarde = 35 / 43</t>
+          <t>Lectura 2: 31 en tiempo + 5 tarde = 36 / 43</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: ✗      S02: ✓      L2: tarde</t>
+          <t>P00: ✗      S02: ✓      L2: ✓</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3214,7 @@
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: ✗      L2: ✗</t>
+          <t>P00: ✓      S02: ✗      L2: tarde</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corte de SD: una baja fuera de los totales (42 activos)
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S02-corte-07sep.xlsx
+++ b/calificaciones/P00-S02-corte-07sep.xlsx
@@ -31,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -91,6 +91,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="001F3864"/>
       <sz val="12"/>
     </font>
@@ -123,7 +129,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -143,6 +149,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
   </fills>
@@ -172,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -199,18 +210,21 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -881,26 +895,26 @@
           <t>320237012</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>BAJA</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>BAJA</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
           <t>—</t>
@@ -908,7 +922,7 @@
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>Sin entregas en el repositorio. Tu lectura si esta registrada.</t>
+          <t>Baja.</t>
         </is>
       </c>
     </row>
@@ -2245,44 +2259,44 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="12" t="inlineStr">
-        <is>
-          <t>Resumen del grupo (43 alumnos)</t>
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>Resumen del grupo (42 alumnos activos · 1 baja no contada)</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="13" t="inlineStr">
-        <is>
-          <t>P00 entregada: 38 / 43   (de esas, 4 sin el nombre adentro)</t>
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>P00 entregada: 38 / 42   (de esas, 4 sin el nombre adentro)</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="13" t="inlineStr">
-        <is>
-          <t>S02 completa: 32 / 43   ·   parcial: 7   ·   sin entregar: 4</t>
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>S02 completa: 32 / 42   ·   parcial: 7   ·   sin entregar: 3</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="13" t="inlineStr">
-        <is>
-          <t>Lectura 2: 31 en tiempo + 5 tarde = 36 / 43</t>
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>Lectura 2: 30 en tiempo + 5 tarde = 35 / 42</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="13" t="inlineStr">
-        <is>
-          <t>Lectura 3 (abierta hasta el 13-sep): 1 / 43</t>
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>Lectura 3 (abierta hasta el 13-sep): 1 / 42</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="13" t="inlineStr">
-        <is>
-          <t>Sin absolutamente nada: 2 / 43</t>
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>Sin absolutamente nada: 2 / 42</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2319,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Correccion · 320250648</t>
         </is>
@@ -2319,99 +2333,99 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>P00: sin nombre      S02: ✓      L2: ✓</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Tu p00 no lleva tu nombre.</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Abrelo, escribe tu nombre completo y haz push.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Tu carpeta se llama Salgado_Roman con mayusculas.</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Deberia ir en minusculas: apellido_nombre.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2436,7 +2450,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Correccion · 319659852</t>
         </is>
@@ -2450,111 +2464,111 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>P00: ✗      S02: parcial      L2: ✗</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Falta el error de puerto ocupado: no aparece en tu evidencia.</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Levanta dos contenedores en el mismo puerto; el segundo falla con 'port is already allocated'. Pega ese texto.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>No tienes p00.</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Crea entregas/tu_carpeta/p00/prueba.txt con tu nombre completo y haz push.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Tu Dockerfile es el unico sin EXPOSE 80.</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>Construye igual, pero agregalo: documenta que el contenedor escucha en el 80.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2579,7 +2593,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Correccion · 320229264</t>
         </is>
@@ -2593,111 +2607,111 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>P00: ✓      S02: parcial      L2: ✗</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>El docker ps que pegaste no muestra tus contenedores: salen miweb, web1 y web2, no los tuyos. La mision 3 se queda sin evidencia.</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Levanta TUS dos contenedores con --name sitio y --name sitio2, corre docker ps y pega esa salida.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>El error de puerto lo describes con tus palabras ('Docker mostro un error equivalente al siguiente') en vez de pegarlo.</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Reproducelo y pega el texto tal cual sale en tu terminal.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Tu index.html no trae la tabla de 5 comandos.</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>Esa era la mision 1: agregala.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2722,7 +2736,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Correccion · 320284858</t>
         </is>
@@ -2736,87 +2750,87 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>P00: sin nombre      S02: ✓      L2: ✗</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Tu p00 dice solo 'prueba', sin tu nombre.</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Abrelo, escribe tu nombre completo y haz push. Tu S02 esta completa.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2841,7 +2855,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Correccion · 320224159</t>
         </is>
@@ -2855,87 +2869,87 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>P00: ✓      S02: parcial      L2: ✓</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Tu evidencia.md esta cortada a la mitad: son 516 caracteres y termina a media instruccion, despues de la lista de comandos.</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Falta el docker ps, el error de puerto ocupado y las dos respuestas. Probablemente no guardaste antes de subir: completala y vuelve a hacer push.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2960,7 +2974,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Correccion · 320049376</t>
         </is>
@@ -2974,87 +2988,87 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>P00: ✗      S02: ✓      L2: ✓</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>No tienes p00, que era la primera tarea de Git.</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Crea entregas/tu_carpeta/p00/prueba.txt con tu nombre completo adentro y haz push. Tu S02 si esta completa.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3079,7 +3093,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Correccion · 423054589</t>
         </is>
@@ -3093,87 +3107,87 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>P00: ✓      S02: parcial      L2: ✓</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Tu index.html todavia dice 'Hola, soy Tu Nombre': es el texto de ejemplo de la guia, no lo cambiaste. Esa era la mision 1.</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Abre tu index.html, pon tu nombre real y vuelve a construir la imagen: docker build -t mi-sitio . y levanta el contenedor otra vez.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3198,7 +3212,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Correccion · 321132477</t>
         </is>
@@ -3212,99 +3226,99 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>P00: ✓      S02: ✗      L2: tarde</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>No subiste nada de la S02: falta el Dockerfile, el index.html y la evidencia.md.</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>La guia del lab esta en labs/Lab-S02-Docker-dia-1.html. Aunque sea tarde, subela: tarde no baja puntos, pero sin entrega no hay calificacion.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Tu p00 esta guardado en latin-1 y tu apellido con ñ sale roto.</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Vuelve a guardarlo eligiendo codificacion UTF-8.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3329,7 +3343,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Correccion · 320298835</t>
         </is>
@@ -3343,99 +3357,99 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>P00: sin nombre      S02: ✓      L2: ✓</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Tu p00 no lleva tu nombre: dice 'esta es una prueba de git'.</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Abrelo, escribe tu nombre completo y haz push.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>En tu evidencia escribes docker build -t mi-sitio sin el punto final.</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>El punto es obligatorio: le dice a Docker donde buscar el Dockerfile.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3460,7 +3474,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Correccion · 117003136</t>
         </is>
@@ -3474,99 +3488,99 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>P00: ✓      S02: parcial      L2: tarde</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="56" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>El error que pegaste no es el que pedia la mision: pegaste 'Conflict. The container name /sitio is already in use', que es de nombre repetido. El que se pedia es el de PUERTO ocupado.</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Levanta dos contenedores en el MISMO puerto: docker run -d -p 9090:80 --name a mi-sitio y luego docker run -d -p 9090:80 --name b mi-sitio. El segundo falla con 'port is already allocated': pega ese texto.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Tu archivo se llama Evidencia.md con mayuscula.</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Renombralo a evidencia.md, todo en minusculas.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3591,7 +3605,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Correccion · 320152841</t>
         </is>
@@ -3605,99 +3619,99 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>P00: ✓      S02: ✓      L2: ✗</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Tu respuesta de por que la pagina no cambio esta equivocada: dices que Docker bloquea la imagen.</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>La razon es que la imagen es inmutable: el contenedor sigue corriendo la imagen vieja, y hasta que no reconstruyes con docker build no existe una imagen nueva.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Tu carpeta lleva solo tu apellido.</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Deberia ser apellido_nombre, igual que tu rama.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3722,7 +3736,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Correccion · 318586465</t>
         </is>
@@ -3736,99 +3750,99 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>P00: ✓      S02: parcial      L2: ✓</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Falta la salida de docker ps (mision 3): no aparece en tu evidencia.</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Con tus dos contenedores corriendo, ejecuta docker ps y pega la salida COMPLETA en tu evidencia.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Tu archivo se llama evindecia.md.</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>Renombralo a evidencia.md.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3853,7 +3867,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Correccion · 320018277</t>
         </is>
@@ -3867,87 +3881,87 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>P00: ✓      S02: parcial      L2: ✓</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="56" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Tu evidencia trae el texto de ejemplo de la guia sin llenar: bajo Mision 3 dice literalmente '[Aqui va el texto que te salio cuando hiciste docker ps]'. Nunca pegaste tu salida real.</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Corre docker ps con tus contenedores arriba y sustituye ese renglon por lo que te salga. Lo que se califica es tu evidencia, no la plantilla.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3972,7 +3986,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Correccion · 320229594</t>
         </is>
@@ -3986,99 +4000,99 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>P00: sin nombre      S02: ✓      L2: ✓</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Tu p00 no lleva tu nombre: dice 'Esta es una prueba de git'.</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>Abrelo, escribe tu nombre completo y haz push.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Escribes docker build -t mi-sitio-v2 sin el punto final, y usas mi-sitio-v2 como si fuera la version 2.</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>El punto es obligatorio: dice donde esta el Dockerfile. Y la version 2 se marca con dos puntos: mi-sitio:v2, no con guion.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>

</xml_diff>

<commit_message>
Corte SD: alta de la lista nueva, lectura atribuida a su autor real y baja fuera de totales
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S02-corte-07sep.xlsx
+++ b/calificaciones/P00-S02-corte-07sep.xlsx
@@ -590,7 +590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1539,9 +1539,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E30" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>Completa. A tu evidencia le falta un encabezado con tu nombre.</t>
+          <t>Completa, y tu lectura si quedo registrada en tiempo. A tu evidencia le falta un encabezado con tu nombre.</t>
         </is>
       </c>
     </row>
@@ -1743,17 +1743,17 @@
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>320250648</t>
-        </is>
-      </c>
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>sin nombre</t>
-        </is>
-      </c>
-      <c r="C36" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
+          <t>318026644</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="D36" s="9" t="inlineStr">
@@ -1761,9 +1761,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="F36" s="9" t="inlineStr">
@@ -1773,24 +1773,24 @@
       </c>
       <c r="G36" s="10" t="inlineStr">
         <is>
-          <t>Completa. Tu p00 no lleva tu nombre y tu carpeta usa mayusculas.</t>
+          <t>Alta reciente. Acepta la invitacion al repositorio para poder entregar: tu rama ya esta lista.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>319659852</t>
-        </is>
-      </c>
-      <c r="B37" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="C37" s="8" t="inlineStr">
-        <is>
-          <t>parcial</t>
+          <t>320250648</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>sin nombre</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
@@ -1798,9 +1798,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E37" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
@@ -1810,34 +1810,34 @@
       </c>
       <c r="G37" s="10" t="inlineStr">
         <is>
-          <t>Subiste tu S02. Falta el error de puerto ocupado, y te falta la p00. Ver tu hoja.</t>
+          <t>Completa. Tu p00 no lleva tu nombre y tu carpeta usa mayusculas.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>320187072</t>
-        </is>
-      </c>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D38" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
+          <t>319659852</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>parcial</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="F38" s="9" t="inlineStr">
@@ -1847,14 +1847,14 @@
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>Completa y correcta.</t>
+          <t>Subiste tu S02. Falta el error de puerto ocupado, y te falta la p00. Ver tu hoja.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>320229264</t>
+          <t>320187072</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -1862,19 +1862,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>parcial</t>
-        </is>
-      </c>
-      <c r="D39" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E39" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F39" s="9" t="inlineStr">
@@ -1884,14 +1884,14 @@
       </c>
       <c r="G39" s="10" t="inlineStr">
         <is>
-          <t>Tu docker ps no corresponde a tus contenedores y falta la tabla de comandos. Ver tu hoja.</t>
+          <t>Completa y correcta.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>320227442</t>
+          <t>320229264</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -1899,9 +1899,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>parcial</t>
         </is>
       </c>
       <c r="D40" s="9" t="inlineStr">
@@ -1909,9 +1909,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="F40" s="9" t="inlineStr">
@@ -1921,19 +1921,19 @@
       </c>
       <c r="G40" s="10" t="inlineStr">
         <is>
-          <t>Completa y correcta.</t>
+          <t>Tu docker ps no corresponde a tus contenedores y falta la tabla de comandos. Ver tu hoja.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>320284858</t>
-        </is>
-      </c>
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>sin nombre</t>
+          <t>320227442</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
@@ -1946,9 +1946,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E41" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F41" s="9" t="inlineStr">
@@ -1958,24 +1958,24 @@
       </c>
       <c r="G41" s="10" t="inlineStr">
         <is>
-          <t>Completa. Tu p00 no lleva tu nombre.</t>
+          <t>Completa y correcta.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>320224159</t>
-        </is>
-      </c>
-      <c r="B42" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t>parcial</t>
+          <t>320284858</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>sin nombre</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="D42" s="9" t="inlineStr">
@@ -1983,9 +1983,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="F42" s="9" t="inlineStr">
@@ -1995,14 +1995,14 @@
       </c>
       <c r="G42" s="10" t="inlineStr">
         <is>
-          <t>Tu evidencia quedo cortada a la mitad. Ver tu hoja.</t>
+          <t>Completa. Tu p00 no lleva tu nombre.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>320301238</t>
+          <t>320224159</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -2010,9 +2010,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>parcial</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
@@ -2032,14 +2032,14 @@
       </c>
       <c r="G43" s="10" t="inlineStr">
         <is>
-          <t>Completa. Tu evidencia tiene los acentos rotos; guardala como UTF-8.</t>
+          <t>Tu evidencia quedo cortada a la mitad. Ver tu hoja.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>317042333</t>
+          <t>320301238</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -2069,14 +2069,14 @@
       </c>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>Completa. Tu evidencia quedo dentro de un bloque de codigo sin cerrar.</t>
+          <t>Completa. Tu evidencia tiene los acentos rotos; guardala como UTF-8.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>312137760</t>
+          <t>317042333</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -2089,9 +2089,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -2106,14 +2106,14 @@
       </c>
       <c r="G45" s="10" t="inlineStr">
         <is>
-          <t>Completa y correcta.</t>
+          <t>Completa. Tu evidencia quedo dentro de un bloque de codigo sin cerrar.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>318259624</t>
+          <t>312137760</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -2126,9 +2126,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D46" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
@@ -2143,14 +2143,14 @@
       </c>
       <c r="G46" s="10" t="inlineStr">
         <is>
-          <t>Completa. Tu docker ps esta recortado; pegalo completo.</t>
+          <t>Completa y correcta.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>423035119</t>
+          <t>318259624</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -2163,9 +2163,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
@@ -2180,14 +2180,14 @@
       </c>
       <c r="G47" s="10" t="inlineStr">
         <is>
-          <t>Completa. Una linea de comandos quedo corrupta al pegar.</t>
+          <t>Completa. Tu docker ps esta recortado; pegalo completo.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>320490572</t>
+          <t>423035119</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -2200,9 +2200,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D48" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
@@ -2210,93 +2210,130 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="G48" s="10" t="inlineStr">
         <is>
-          <t>Completa. Usaste tags propios en vez de mi-sitio.</t>
+          <t>Completa. Una linea de comandos quedo corrupta al pegar.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
+          <t>320490572</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G49" s="10" t="inlineStr">
+        <is>
+          <t>Completa. Usaste tags propios en vez de mi-sitio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
           <t>320049376</t>
         </is>
       </c>
-      <c r="B49" s="11" t="inlineStr">
+      <c r="B50" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="C49" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="D49" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E49" s="7" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="F49" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G49" s="10" t="inlineStr">
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G50" s="10" t="inlineStr">
         <is>
           <t>Tu S02 esta completa y tu lectura entro en tiempo. Falta tu p00.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>Resumen del grupo (42 alumnos activos · 1 baja no contada)</t>
-        </is>
-      </c>
-    </row>
     <row r="52">
-      <c r="A52" s="14" t="inlineStr">
-        <is>
-          <t>P00 entregada: 38 / 42   (de esas, 4 sin el nombre adentro)</t>
+      <c r="A52" s="13" t="inlineStr">
+        <is>
+          <t>Resumen del grupo (43 alumnos activos · 1 baja no contada)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="14" t="inlineStr">
         <is>
-          <t>S02 completa: 32 / 42   ·   parcial: 7   ·   sin entregar: 3</t>
+          <t>P00 entregada: 38 / 43   (de esas, 4 sin el nombre adentro)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="14" t="inlineStr">
         <is>
-          <t>Lectura 2: 30 en tiempo + 5 tarde = 35 / 42</t>
+          <t>S02 completa: 32 / 43   ·   parcial: 7   ·   sin entregar: 4</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
         <is>
-          <t>Lectura 3 (abierta hasta el 13-sep): 1 / 42</t>
+          <t>Lectura 2: 31 en tiempo + 5 tarde = 36 / 43</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="14" t="inlineStr">
         <is>
-          <t>Sin absolutamente nada: 2 / 42</t>
+          <t>Lectura 3 (abierta hasta el 13-sep): 1 / 43</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="14" t="inlineStr">
+        <is>
+          <t>Sin absolutamente nada: 3 / 43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corte SD: una p00 entregada hoy y su s02 aceptada
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S02-corte-07sep.xlsx
+++ b/calificaciones/P00-S02-corte-07sep.xlsx
@@ -17,11 +17,10 @@
     <sheet name="320018277" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="320229594" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="320250648" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="319659852" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="320229264" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="320284858" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="320224159" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="320049376" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="320229264" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="320284858" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="320224159" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="320049376" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1820,26 +1819,26 @@
           <t>319659852</t>
         </is>
       </c>
-      <c r="B38" s="11" t="inlineStr">
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>parcial</t>
-        </is>
-      </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E38" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
           <t>—</t>
@@ -1847,7 +1846,7 @@
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>Subiste tu S02. Falta el error de puerto ocupado, y te falta la p00. Ver tu hoja.</t>
+          <t>Completa. Tu p00 quedo registrada y tu S02 cuenta como entregada.</t>
         </is>
       </c>
     </row>
@@ -2305,14 +2304,14 @@
     <row r="53">
       <c r="A53" s="14" t="inlineStr">
         <is>
-          <t>P00 entregada: 38 / 43   (de esas, 4 sin el nombre adentro)</t>
+          <t>P00 entregada: 39 / 43   (de esas, 4 sin el nombre adentro)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="14" t="inlineStr">
         <is>
-          <t>S02 completa: 32 / 43   ·   parcial: 7   ·   sin entregar: 4</t>
+          <t>S02 completa: 33 / 43   ·   parcial: 6   ·   sin entregar: 4</t>
         </is>
       </c>
     </row>
@@ -2489,21 +2488,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 319659852</t>
+          <t>Correccion · 320229264</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 319659852   ·   Por corregir: S02 y p00</t>
+          <t>Cuenta: 320229264   ·   Por corregir: S02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: ✗      S02: parcial      L2: ✗</t>
+          <t>P00: ✓      S02: parcial      L2: ✗</t>
         </is>
       </c>
     </row>
@@ -2522,36 +2521,36 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>Falta el error de puerto ocupado: no aparece en tu evidencia.</t>
+          <t>El docker ps que pegaste no muestra tus contenedores: salen miweb, web1 y web2, no los tuyos. La mision 3 se queda sin evidencia.</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Levanta dos contenedores en el mismo puerto; el segundo falla con 'port is already allocated'. Pega ese texto.</t>
+          <t>Levanta TUS dos contenedores con --name sitio y --name sitio2, corre docker ps y pega esa salida.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>No tienes p00.</t>
+          <t>El error de puerto lo describes con tus palabras ('Docker mostro un error equivalente al siguiente') en vez de pegarlo.</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Crea entregas/tu_carpeta/p00/prueba.txt con tu nombre completo y haz push.</t>
+          <t>Reproducelo y pega el texto tal cual sale en tu terminal.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>Tu Dockerfile es el unico sin EXPOSE 80.</t>
+          <t>Tu index.html no trae la tabla de 5 comandos.</t>
         </is>
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>Construye igual, pero agregalo: documenta que el contenedor escucha en el 80.</t>
+          <t>Esa era la mision 1: agregala.</t>
         </is>
       </c>
     </row>
@@ -2622,7 +2621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -2632,21 +2631,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 320229264</t>
+          <t>Correccion · 320284858</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320229264   ·   Por corregir: S02</t>
+          <t>Cuenta: 320284858   ·   Por corregir: p00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: parcial      L2: ✗</t>
+          <t>P00: sin nombre      S02: ✓      L2: ✗</t>
         </is>
       </c>
     </row>
@@ -2665,90 +2664,66 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>El docker ps que pegaste no muestra tus contenedores: salen miweb, web1 y web2, no los tuyos. La mision 3 se queda sin evidencia.</t>
+          <t>Tu p00 dice solo 'prueba', sin tu nombre.</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Levanta TUS dos contenedores con --name sitio y --name sitio2, corre docker ps y pega esa salida.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>El error de puerto lo describes con tus palabras ('Docker mostro un error equivalente al siguiente') en vez de pegarlo.</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Reproducelo y pega el texto tal cual sale en tu terminal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
-        <is>
-          <t>Tu index.html no trae la tabla de 5 comandos.</t>
-        </is>
-      </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>Esa era la mision 1: agregala.</t>
+          <t>Abrelo, escribe tu nombre completo y haz push. Tu S02 esta completa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>git checkout TU-RAMA</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
+          <t>git push</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2775,21 +2750,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 320284858</t>
+          <t>Correccion · 320224159</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320284858   ·   Por corregir: p00</t>
+          <t>Cuenta: 320224159   ·   Por corregir: S02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: sin nombre      S02: ✓      L2: ✗</t>
+          <t>P00: ✓      S02: parcial      L2: ✓</t>
         </is>
       </c>
     </row>
@@ -2808,12 +2783,12 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>Tu p00 dice solo 'prueba', sin tu nombre.</t>
+          <t>Tu evidencia.md esta cortada a la mitad: son 516 caracteres y termina a media instruccion, despues de la lista de comandos.</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Abrelo, escribe tu nombre completo y haz push. Tu S02 esta completa.</t>
+          <t>Falta el docker ps, el error de puerto ocupado y las dos respuestas. Probablemente no guardaste antes de subir: completala y vuelve a hacer push.</t>
         </is>
       </c>
     </row>
@@ -2894,125 +2869,6 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 320224159</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 320224159   ·   Por corregir: S02</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: ✓      S02: parcial      L2: ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Tu evidencia.md esta cortada a la mitad: son 516 caracteres y termina a media instruccion, despues de la lista de comandos.</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Falta el docker ps, el error de puerto ocupado y las dos respuestas. Probablemente no guardaste antes de subir: completala y vuelve a hacer push.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
           <t>Correccion · 320049376</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Corte SD: s02 aceptada con sus dos correcciones aun pendientes
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S02-corte-07sep.xlsx
+++ b/calificaciones/P00-S02-corte-07sep.xlsx
@@ -17,10 +17,11 @@
     <sheet name="320018277" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="320229594" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="320250648" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="320229264" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="320284858" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="320224159" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="320049376" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="319659852" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="320229264" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="320284858" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="320224159" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="320049376" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1846,7 +1847,7 @@
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
-          <t>Completa. Tu p00 quedo registrada y tu S02 cuenta como entregada.</t>
+          <t>Tu p00 quedo registrada y tu S02 ya cuenta como entregada. Te faltan las dos correcciones de tu hoja.</t>
         </is>
       </c>
     </row>
@@ -2488,21 +2489,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 320229264</t>
+          <t>Correccion · 319659852</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320229264   ·   Por corregir: S02</t>
+          <t>Cuenta: 319659852   ·   Por corregir: S02 · lo que quedaste de corregir</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: parcial      L2: ✗</t>
+          <t>P00: ✓      S02: ✓      L2: ✗</t>
         </is>
       </c>
     </row>
@@ -2521,36 +2522,36 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>El docker ps que pegaste no muestra tus contenedores: salen miweb, web1 y web2, no los tuyos. La mision 3 se queda sin evidencia.</t>
+          <t>Falta el error de puerto ocupado: no aparece en tu evidencia.</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Levanta TUS dos contenedores con --name sitio y --name sitio2, corre docker ps y pega esa salida.</t>
+          <t>Levanta dos contenedores en el mismo puerto; el segundo falla con 'port is already allocated'. Pega ese texto en tu evidencia.md.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>El error de puerto lo describes con tus palabras ('Docker mostro un error equivalente al siguiente') en vez de pegarlo.</t>
+          <t>Tu Dockerfile es el unico sin EXPOSE 80.</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Reproducelo y pega el texto tal cual sale en tu terminal.</t>
+          <t>Agregale la linea EXPOSE 80 . Construye igual, pero documenta que el contenedor escucha en ese puerto.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>Tu index.html no trae la tabla de 5 comandos.</t>
+          <t>Tu p00 ya quedo registrada, esa ya no le muevas.</t>
         </is>
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>Esa era la mision 1: agregala.</t>
+          <t>Tu S02 ya cuenta como entregada: estas dos correcciones son para dejarla completa.</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -2631,21 +2632,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 320284858</t>
+          <t>Correccion · 320229264</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320284858   ·   Por corregir: p00</t>
+          <t>Cuenta: 320229264   ·   Por corregir: S02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: sin nombre      S02: ✓      L2: ✗</t>
+          <t>P00: ✓      S02: parcial      L2: ✗</t>
         </is>
       </c>
     </row>
@@ -2664,66 +2665,90 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>Tu p00 dice solo 'prueba', sin tu nombre.</t>
+          <t>El docker ps que pegaste no muestra tus contenedores: salen miweb, web1 y web2, no los tuyos. La mision 3 se queda sin evidencia.</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Abrelo, escribe tu nombre completo y haz push. Tu S02 esta completa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+          <t>Levanta TUS dos contenedores con --name sitio y --name sitio2, corre docker ps y pega esa salida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>El error de puerto lo describes con tus palabras ('Docker mostro un error equivalente al siguiente') en vez de pegarlo.</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Reproducelo y pega el texto tal cual sale en tu terminal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Tu index.html no trae la tabla de 5 comandos.</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Esa era la mision 1: agregala.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>git commit -m "S02: correccion"</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>git commit -m "S02: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
           <t>git push</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2750,21 +2775,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 320224159</t>
+          <t>Correccion · 320284858</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320224159   ·   Por corregir: S02</t>
+          <t>Cuenta: 320284858   ·   Por corregir: p00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: parcial      L2: ✓</t>
+          <t>P00: sin nombre      S02: ✓      L2: ✗</t>
         </is>
       </c>
     </row>
@@ -2783,12 +2808,12 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>Tu evidencia.md esta cortada a la mitad: son 516 caracteres y termina a media instruccion, despues de la lista de comandos.</t>
+          <t>Tu p00 dice solo 'prueba', sin tu nombre.</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Falta el docker ps, el error de puerto ocupado y las dos respuestas. Probablemente no guardaste antes de subir: completala y vuelve a hacer push.</t>
+          <t>Abrelo, escribe tu nombre completo y haz push. Tu S02 esta completa.</t>
         </is>
       </c>
     </row>
@@ -2869,6 +2894,125 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
+          <t>Correccion · 320224159</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 320224159   ·   Por corregir: S02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>P00: ✓      S02: parcial      L2: ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Tu evidencia.md esta cortada a la mitad: son 516 caracteres y termina a media instruccion, despues de la lista de comandos.</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Falta el docker ps, el error de puerto ocupado y las dos respuestas. Probablemente no guardaste antes de subir: completala y vuelve a hacer push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>git commit -m "S02: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
           <t>Correccion · 320049376</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Corte SD: P00 cuenta para todo el que hizo push, y se registran dos correcciones
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S02-corte-07sep.xlsx
+++ b/calificaciones/P00-S02-corte-07sep.xlsx
@@ -14,14 +14,12 @@
     <sheet name="117003136" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="320152841" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="318586465" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="320018277" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="320229594" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="320250648" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="319659852" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="320229264" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="320284858" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="320224159" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="320049376" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="320250648" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="319659852" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="320229264" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="320284858" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="320224159" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="320049376" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -619,7 +617,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>✓ = completa  ·  parcial = le falta algo (ver tu hoja)  ·  sin nombre = entregada pero el archivo no te identifica  ·  ✗ = no entregada  ·  tarde = fuera de tiempo, no baja puntos</t>
+          <t>✓ = completa  ·  parcial = le falta algo (ver tu hoja)  ·  ✗ = no entregada  ·  tarde = fuera de tiempo, no baja puntos.  P00: el objetivo era demostrar que sabes hacer push, asi que cuenta para todo el que subio algo.</t>
         </is>
       </c>
     </row>
@@ -710,26 +708,26 @@
           <t>423035470</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
           <t>—</t>
@@ -737,7 +735,7 @@
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>Sin entregas registradas.</t>
+          <t>Ya hiciste tu primer push. Falta toda la S02.</t>
         </is>
       </c>
     </row>
@@ -821,9 +819,9 @@
           <t>320298835</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>sin nombre</t>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -848,7 +846,7 @@
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>Completa. Tu p00 no lleva tu nombre y en la evidencia falta el punto de contexto del build.</t>
+          <t>Completa. Detalle: en la evidencia falta el punto de contexto del build.</t>
         </is>
       </c>
     </row>
@@ -996,7 +994,7 @@
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>Completa. Tu p00 quedo en UTF-16; guardalo como UTF-8.</t>
+          <t>Completa y correcta.</t>
         </is>
       </c>
     </row>
@@ -1455,9 +1453,9 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>parcial</t>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
@@ -1477,7 +1475,7 @@
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>Tu evidencia trae el texto de ejemplo de la guia sin llenar. Ver tu hoja.</t>
+          <t>Corregida y aceptada: tu docker ps real ya quedo en tu evidencia.</t>
         </is>
       </c>
     </row>
@@ -1709,9 +1707,9 @@
           <t>320229594</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>sin nombre</t>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -1736,7 +1734,7 @@
       </c>
       <c r="G35" s="10" t="inlineStr">
         <is>
-          <t>Completa. Tu p00 no lleva tu nombre y confundiste el tag v2. Ver tu hoja.</t>
+          <t>Completa. Tu p00 ya quedo corregida. Detalle: confundiste el tag v2.</t>
         </is>
       </c>
     </row>
@@ -1783,9 +1781,9 @@
           <t>320250648</t>
         </is>
       </c>
-      <c r="B37" s="8" t="inlineStr">
-        <is>
-          <t>sin nombre</t>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
@@ -1810,7 +1808,7 @@
       </c>
       <c r="G37" s="10" t="inlineStr">
         <is>
-          <t>Completa. Tu p00 no lleva tu nombre y tu carpeta usa mayusculas.</t>
+          <t>Completa y correcta.</t>
         </is>
       </c>
     </row>
@@ -1968,9 +1966,9 @@
           <t>320284858</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
-        <is>
-          <t>sin nombre</t>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
@@ -1995,7 +1993,7 @@
       </c>
       <c r="G42" s="10" t="inlineStr">
         <is>
-          <t>Completa. Tu p00 no lleva tu nombre.</t>
+          <t>Completa y correcta.</t>
         </is>
       </c>
     </row>
@@ -2264,9 +2262,9 @@
           <t>320049376</t>
         </is>
       </c>
-      <c r="B50" s="11" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
@@ -2291,7 +2289,7 @@
       </c>
       <c r="G50" s="10" t="inlineStr">
         <is>
-          <t>Tu S02 esta completa y tu lectura entro en tiempo. Falta tu p00.</t>
+          <t>Completa y correcta, y tu lectura entro en tiempo.</t>
         </is>
       </c>
     </row>
@@ -2305,14 +2303,14 @@
     <row r="53">
       <c r="A53" s="14" t="inlineStr">
         <is>
-          <t>P00 entregada: 39 / 43   (de esas, 4 sin el nombre adentro)</t>
+          <t>P00 entregada: 41 / 43   (de esas, 0 sin el nombre adentro)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="14" t="inlineStr">
         <is>
-          <t>S02 completa: 33 / 43   ·   parcial: 6   ·   sin entregar: 4</t>
+          <t>S02 completa: 34 / 43   ·   parcial: 5   ·   sin entregar: 4</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2331,7 @@
     <row r="57">
       <c r="A57" s="14" t="inlineStr">
         <is>
-          <t>Sin absolutamente nada: 3 / 43</t>
+          <t>Sin absolutamente nada: 2 / 43</t>
         </is>
       </c>
     </row>
@@ -2343,137 +2341,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>Correccion · 320250648</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 320250648   ·   Por corregir: p00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: sin nombre      S02: ✓      L2: ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Tu p00 no lleva tu nombre.</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Abrelo, escribe tu nombre completo y haz push.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>Tu carpeta se llama Salgado_Roman con mayusculas.</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Deberia ir en minusculas: apellido_nombre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2489,21 +2356,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 319659852</t>
+          <t>Correccion · 320229264</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 319659852   ·   Por corregir: S02 · lo que quedaste de corregir</t>
+          <t>Cuenta: 320229264   ·   Por corregir: S02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: ✓      L2: ✗</t>
+          <t>P00: ✓      S02: parcial      L2: ✗</t>
         </is>
       </c>
     </row>
@@ -2522,36 +2389,36 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>Falta el error de puerto ocupado: no aparece en tu evidencia.</t>
+          <t>El docker ps que pegaste no muestra tus contenedores: salen miweb, web1 y web2, no los tuyos. La mision 3 se queda sin evidencia.</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Levanta dos contenedores en el mismo puerto; el segundo falla con 'port is already allocated'. Pega ese texto en tu evidencia.md.</t>
+          <t>Levanta TUS dos contenedores con --name sitio y --name sitio2, corre docker ps y pega esa salida.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>Tu Dockerfile es el unico sin EXPOSE 80.</t>
+          <t>El error de puerto lo describes con tus palabras ('Docker mostro un error equivalente al siguiente') en vez de pegarlo.</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Agregale la linea EXPOSE 80 . Construye igual, pero documenta que el contenedor escucha en ese puerto.</t>
+          <t>Reproducelo y pega el texto tal cual sale en tu terminal.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>Tu p00 ya quedo registrada, esa ya no le muevas.</t>
+          <t>Tu index.html no trae la tabla de 5 comandos.</t>
         </is>
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>Tu S02 ya cuenta como entregada: estas dos correcciones son para dejarla completa.</t>
+          <t>Esa era la mision 1: agregala.</t>
         </is>
       </c>
     </row>
@@ -2606,6 +2473,125 @@
     </row>
     <row r="17">
       <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Correccion · 320284858</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 320284858   ·   Por corregir: p00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>P00: ✓      S02: ✓      L2: ✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Tu p00 dice solo 'prueba', sin tu nombre.</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Abrelo, escribe tu nombre completo y haz push. Tu S02 esta completa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>git commit -m "S02: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2622,7 +2608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -2632,21 +2618,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 320229264</t>
+          <t>Correccion · 320224159</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320229264   ·   Por corregir: S02</t>
+          <t>Cuenta: 320224159   ·   Por corregir: S02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: parcial      L2: ✗</t>
+          <t>P00: ✓      S02: parcial      L2: ✓</t>
         </is>
       </c>
     </row>
@@ -2665,90 +2651,66 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>El docker ps que pegaste no muestra tus contenedores: salen miweb, web1 y web2, no los tuyos. La mision 3 se queda sin evidencia.</t>
+          <t>Tu evidencia.md esta cortada a la mitad: son 516 caracteres y termina a media instruccion, despues de la lista de comandos.</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Levanta TUS dos contenedores con --name sitio y --name sitio2, corre docker ps y pega esa salida.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>El error de puerto lo describes con tus palabras ('Docker mostro un error equivalente al siguiente') en vez de pegarlo.</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Reproducelo y pega el texto tal cual sale en tu terminal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
-        <is>
-          <t>Tu index.html no trae la tabla de 5 comandos.</t>
-        </is>
-      </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>Esa era la mision 1: agregala.</t>
+          <t>Falta el docker ps, el error de puerto ocupado y las dos respuestas. Probablemente no guardaste antes de subir: completala y vuelve a hacer push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>git checkout TU-RAMA</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
+          <t>git push</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2775,259 +2737,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 320284858</t>
+          <t>Correccion · 320049376</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320284858   ·   Por corregir: p00</t>
+          <t>Cuenta: 320049376   ·   Por corregir: p00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: sin nombre      S02: ✓      L2: ✗</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Tu p00 dice solo 'prueba', sin tu nombre.</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Abrelo, escribe tu nombre completo y haz push. Tu S02 esta completa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>Correccion · 320224159</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 320224159   ·   Por corregir: S02</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: ✓      S02: parcial      L2: ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Tu evidencia.md esta cortada a la mitad: son 516 caracteres y termina a media instruccion, despues de la lista de comandos.</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Falta el docker ps, el error de puerto ocupado y las dos respuestas. Probablemente no guardaste antes de subir: completala y vuelve a hacer push.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>Correccion · 320049376</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 320049376   ·   Por corregir: p00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: ✗      S02: ✓      L2: ✓</t>
+          <t>P00: ✓      S02: ✓      L2: ✓</t>
         </is>
       </c>
     </row>
@@ -3396,7 +3120,7 @@
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: sin nombre      S02: ✓      L2: ✓</t>
+          <t>P00: ✓      S02: ✓      L2: ✓</t>
         </is>
       </c>
     </row>
@@ -3896,7 +3620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -3906,21 +3630,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 320018277</t>
+          <t>Correccion · 320250648</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320018277   ·   Por corregir: S02</t>
+          <t>Cuenta: 320250648   ·   Por corregir: p00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: parcial      L2: ✓</t>
+          <t>P00: ✓      S02: ✓      L2: ✓</t>
         </is>
       </c>
     </row>
@@ -3936,69 +3660,81 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="56" customHeight="1">
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>Tu evidencia trae el texto de ejemplo de la guia sin llenar: bajo Mision 3 dice literalmente '[Aqui va el texto que te salio cuando hiciste docker ps]'. Nunca pegaste tu salida real.</t>
+          <t>Tu p00 no lleva tu nombre.</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Corre docker ps con tus contenedores arriba y sustituye ese renglon por lo que te salga. Lo que se califica es tu evidencia, no la plantilla.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+          <t>Abrelo, escribe tu nombre completo y haz push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Tu carpeta se llama Salgado_Roman con mayusculas.</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Deberia ir en minusculas: apellido_nombre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>git commit -m "S02: correccion"</t>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
+          <t>git commit -m "S02: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
           <t>git push</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -4015,7 +3751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -4025,21 +3761,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 320229594</t>
+          <t>Correccion · 319659852</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320229594   ·   Por corregir: S02 y p00</t>
+          <t>Cuenta: 319659852   ·   Por corregir: S02 · lo que quedaste de corregir</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: sin nombre      S02: ✓      L2: ✓</t>
+          <t>P00: ✓      S02: ✓      L2: ✗</t>
         </is>
       </c>
     </row>
@@ -4058,78 +3794,90 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>Tu p00 no lleva tu nombre: dice 'Esta es una prueba de git'.</t>
+          <t>Falta el error de puerto ocupado: no aparece en tu evidencia.</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Abrelo, escribe tu nombre completo y haz push.</t>
+          <t>Levanta dos contenedores en el mismo puerto; el segundo falla con 'port is already allocated'. Pega ese texto en tu evidencia.md.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>Escribes docker build -t mi-sitio-v2 sin el punto final, y usas mi-sitio-v2 como si fuera la version 2.</t>
+          <t>Tu Dockerfile es el unico sin EXPOSE 80.</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>El punto es obligatorio: dice donde esta el Dockerfile. Y la version 2 se marca con dos puntos: mi-sitio:v2, no con guion.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+          <t>Agregale la linea EXPOSE 80 . Construye igual, pero documenta que el contenedor escucha en ese puerto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Tu p00 ya quedo registrada, esa ya no le muevas.</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Tu S02 ya cuenta como entregada: estas dos correcciones son para dejarla completa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
-          <t>git commit -m "S02: correccion"</t>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="19" t="inlineStr">
         <is>
+          <t>git commit -m "S02: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
           <t>git push</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>

</xml_diff>

<commit_message>
Corte SD: agrega la columna de la tarea opcional
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S02-corte-07sep.xlsx
+++ b/calificaciones/P00-S02-corte-07sep.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -597,7 +597,8 @@
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="74" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -624,7 +625,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>L1 era opcional. L2 cerro el sabado 06-sep 06:59 (tarde: hasta el domingo). L3 sigue abierta hasta el sabado 13-sep 06:59. El lab de la S03 no venia en este corte.</t>
+          <t>L1 era opcional. L2 cerro el sabado 06-sep 06:59 (tarde: hasta el domingo). L3 sigue abierta hasta el sabado 13-sep 06:59. Opcional = la tarea opcional de idempotency key (entregas/OPCIONALES.md): no afecta tu calificacion, cuenta para los puntos extra del final.</t>
         </is>
       </c>
     </row>
@@ -661,6 +662,11 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
+          <t>Opcional</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
           <t>Observaciones</t>
         </is>
       </c>
@@ -696,7 +702,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
         <is>
           <t>Tu index.html quedo con el nombre de ejemplo de la guia. Ver tu hoja.</t>
         </is>
@@ -733,7 +744,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G8" s="10" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
         <is>
           <t>Ya hiciste tu primer push. Falta toda la S02.</t>
         </is>
@@ -770,7 +786,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="10" t="inlineStr">
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -807,7 +828,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G10" s="10" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>Tus lecturas SI estan registradas. Falta la S02: cuando la subas se actualiza.</t>
         </is>
@@ -844,7 +870,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
         <is>
           <t>Completa. Detalle: en la evidencia falta el punto de contexto del build.</t>
         </is>
@@ -881,7 +912,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G12" s="10" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -918,7 +954,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G13" s="10" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
         <is>
           <t>Baja.</t>
         </is>
@@ -955,7 +996,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G14" s="10" t="inlineStr">
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
         <is>
           <t>Completa. Te quedo un hola_mundo.py suelto en la carpeta.</t>
         </is>
@@ -992,7 +1038,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G15" s="10" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1029,7 +1080,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G16" s="10" t="inlineStr">
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu S02 estaba en una rama vieja; ya la movimos a tu rama.</t>
         </is>
@@ -1066,7 +1122,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G17" s="10" t="inlineStr">
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
         <is>
           <t>El error que pegaste no es el de puerto ocupado. Ver tu hoja.</t>
         </is>
@@ -1103,7 +1164,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu entrega estaba en tu rama vieja y no la habiamos visto: ya la consolidamos en tu rama. Tu evidencia esta muy bien. Detalle menor: en p00 te quedaron archivos de mas.</t>
         </is>
@@ -1140,7 +1206,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G19" s="10" t="inlineStr">
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
         <is>
           <t>Completa y bien organizada.</t>
         </is>
@@ -1177,7 +1248,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G20" s="10" t="inlineStr">
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
         <is>
           <t>Sin entregas registradas.</t>
         </is>
@@ -1214,7 +1290,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G21" s="10" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu docker ps esta recortado a mano; pegalo tal cual sale.</t>
         </is>
@@ -1251,7 +1332,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G22" s="10" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu S02 estaba en una rama vieja y tu carpeta tenia otro nombre; ya las acomodamos.</t>
         </is>
@@ -1288,7 +1374,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G23" s="10" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1325,7 +1416,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G24" s="10" t="inlineStr">
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu carpeta lleva solo tu apellido, y tu respuesta sobre por que no cambio la pagina no es correcta. Ver tu hoja.</t>
         </is>
@@ -1362,7 +1458,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G25" s="10" t="inlineStr">
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1399,7 +1500,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G26" s="10" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
         <is>
           <t>Completa y muy bien documentada.</t>
         </is>
@@ -1436,7 +1542,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G27" s="10" t="inlineStr">
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
         <is>
           <t>Falta la salida de docker ps. Ver tu hoja.</t>
         </is>
@@ -1473,7 +1584,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G28" s="10" t="inlineStr">
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
         <is>
           <t>Corregida y aceptada: tu docker ps real ya quedo en tu evidencia.</t>
         </is>
@@ -1510,7 +1626,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G29" s="10" t="inlineStr">
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1547,7 +1668,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G30" s="10" t="inlineStr">
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
         <is>
           <t>Completa, y tu lectura si quedo registrada en tiempo. A tu evidencia le falta un encabezado con tu nombre.</t>
         </is>
@@ -1584,7 +1710,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G31" s="10" t="inlineStr">
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
         <is>
           <t>Completa. Listaste docker system prune, que la guia pide no usar.</t>
         </is>
@@ -1621,7 +1752,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G32" s="10" t="inlineStr">
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu archivo deberia llamarse evidencia.md, sin espacios.</t>
         </is>
@@ -1658,7 +1794,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G33" s="10" t="inlineStr">
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H33" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1695,7 +1836,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G34" s="10" t="inlineStr">
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu markdown quedo escapado y se ve en crudo.</t>
         </is>
@@ -1732,7 +1878,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G35" s="10" t="inlineStr">
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu p00 ya quedo corregida. Detalle: confundiste el tag v2.</t>
         </is>
@@ -1769,7 +1920,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G36" s="10" t="inlineStr">
+      <c r="G36" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="10" t="inlineStr">
         <is>
           <t>Alta reciente. Acepta la invitacion al repositorio para poder entregar: tu rama ya esta lista.</t>
         </is>
@@ -1806,7 +1962,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G37" s="10" t="inlineStr">
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1843,7 +2004,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G38" s="10" t="inlineStr">
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H38" s="10" t="inlineStr">
         <is>
           <t>Tu p00 quedo registrada y tu S02 ya cuenta como entregada. Te faltan las dos correcciones de tu hoja.</t>
         </is>
@@ -1880,7 +2046,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G39" s="10" t="inlineStr">
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1917,7 +2088,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G40" s="10" t="inlineStr">
+      <c r="G40" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H40" s="10" t="inlineStr">
         <is>
           <t>Tu docker ps no corresponde a tus contenedores y falta la tabla de comandos. Ver tu hoja.</t>
         </is>
@@ -1954,7 +2130,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G41" s="10" t="inlineStr">
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H41" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1991,7 +2172,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G42" s="10" t="inlineStr">
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H42" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -2028,7 +2214,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G43" s="10" t="inlineStr">
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H43" s="10" t="inlineStr">
         <is>
           <t>Tu evidencia quedo cortada a la mitad. Ver tu hoja.</t>
         </is>
@@ -2065,7 +2256,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G44" s="10" t="inlineStr">
+      <c r="G44" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H44" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu evidencia tiene los acentos rotos; guardala como UTF-8.</t>
         </is>
@@ -2102,7 +2298,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G45" s="10" t="inlineStr">
+      <c r="G45" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H45" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu evidencia quedo dentro de un bloque de codigo sin cerrar.</t>
         </is>
@@ -2139,7 +2340,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G46" s="10" t="inlineStr">
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H46" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -2176,7 +2382,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G47" s="10" t="inlineStr">
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu docker ps esta recortado; pegalo completo.</t>
         </is>
@@ -2213,7 +2424,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G48" s="10" t="inlineStr">
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H48" s="10" t="inlineStr">
         <is>
           <t>Completa. Una linea de comandos quedo corrupta al pegar.</t>
         </is>
@@ -2250,7 +2466,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G49" s="10" t="inlineStr">
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H49" s="10" t="inlineStr">
         <is>
           <t>Completa. Usaste tags propios en vez de mi-sitio.</t>
         </is>
@@ -2287,7 +2508,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G50" s="10" t="inlineStr">
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H50" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta, y tu lectura entro en tiempo.</t>
         </is>
@@ -2332,6 +2558,13 @@
       <c r="A57" s="14" t="inlineStr">
         <is>
           <t>Sin absolutamente nada: 2 / 43</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
+        <is>
+          <t>Tarea opcional (idempotency key): 0 / 43 — sigue abierta, no afecta la calificacion</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corte SD: la columna extra se llama idempotency key, y las S02 con detalles minimos quedan completas
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S02-corte-07sep.xlsx
+++ b/calificaciones/P00-S02-corte-07sep.xlsx
@@ -8,18 +8,15 @@
   </bookViews>
   <sheets>
     <sheet name="Matriz" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="423054589" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="321132477" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="320298835" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="117003136" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="320152841" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="318586465" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="320250648" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="319659852" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="320229264" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="320284858" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="320224159" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="320049376" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="321132477" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="320298835" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="320152841" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="320250648" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="319659852" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="320229264" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="320284858" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="320224159" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="320049376" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -141,12 +138,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
+        <fgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -196,16 +193,16 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -597,8 +594,8 @@
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="66" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -625,7 +622,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>L1 era opcional. L2 cerro el sabado 06-sep 06:59 (tarde: hasta el domingo). L3 sigue abierta hasta el sabado 13-sep 06:59. Opcional = la tarea opcional de idempotency key (entregas/OPCIONALES.md): no afecta tu calificacion, cuenta para los puntos extra del final.</t>
+          <t>L1 era opcional. L2 cerro el sabado 06-sep 06:59 (tarde: hasta el domingo). L3 sigue abierta hasta el sabado 13-sep 06:59. Idempotency key = la tarea EXTRA de entregas/OPCIONALES.md: es opcional, no afecta tu calificacion y cuenta para los puntos extra del final.</t>
         </is>
       </c>
     </row>
@@ -662,7 +659,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Opcional</t>
+          <t>Idempotency key</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -682,12 +679,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>parcial</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -697,19 +694,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>Tu index.html quedo con el nombre de ejemplo de la guia. Ver tu hoja.</t>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>Completa. Detalle: tu index.html se quedo con el nombre de ejemplo de la guia.</t>
         </is>
       </c>
     </row>
@@ -724,32 +721,32 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
         <is>
           <t>Ya hiciste tu primer push. Falta toda la S02.</t>
         </is>
@@ -771,7 +768,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -781,17 +778,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -808,7 +805,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -818,22 +815,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>tarde</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
         <is>
           <t>Tus lecturas SI estan registradas. Falta la S02: cuando la subas se actualiza.</t>
         </is>
@@ -855,7 +852,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -865,17 +862,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>Completa. Detalle: en la evidencia falta el punto de contexto del build.</t>
         </is>
@@ -897,7 +894,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -907,17 +904,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -939,27 +936,27 @@
           <t>BAJA</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>Baja.</t>
         </is>
@@ -981,7 +978,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -991,17 +988,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="9" t="inlineStr">
         <is>
           <t>Completa. Te quedo un hola_mundo.py suelto en la carpeta.</t>
         </is>
@@ -1023,7 +1020,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1033,17 +1030,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1075,17 +1072,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" s="10" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
         <is>
           <t>Completa. Tu S02 estaba en una rama vieja; ya la movimos a tu rama.</t>
         </is>
@@ -1102,34 +1099,34 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>parcial</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>tarde</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H17" s="10" t="inlineStr">
-        <is>
-          <t>El error que pegaste no es el de puerto ocupado. Ver tu hoja.</t>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Completa. Detalle: el error que pegaste no es el de puerto ocupado, sino el de nombre repetido.</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1146,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1159,17 +1156,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" s="10" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
         <is>
           <t>Completa. Tu entrega estaba en tu rama vieja y no la habiamos visto: ya la consolidamos en tu rama. Tu evidencia esta muy bien. Detalle menor: en p00 te quedaron archivos de mas.</t>
         </is>
@@ -1191,7 +1188,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1201,17 +1198,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
         <is>
           <t>Completa y bien organizada.</t>
         </is>
@@ -1223,37 +1220,37 @@
           <t>114001456</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G20" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H20" s="10" t="inlineStr">
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
         <is>
           <t>Sin entregas registradas.</t>
         </is>
@@ -1275,27 +1272,27 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>tarde</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H21" s="10" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
         <is>
           <t>Completa. Tu docker ps esta recortado a mano; pegalo tal cual sale.</t>
         </is>
@@ -1317,7 +1314,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1327,17 +1324,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H22" s="10" t="inlineStr">
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
         <is>
           <t>Completa. Tu S02 estaba en una rama vieja y tu carpeta tenia otro nombre; ya las acomodamos.</t>
         </is>
@@ -1359,7 +1356,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1369,17 +1366,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H23" s="10" t="inlineStr">
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1401,27 +1398,27 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E24" s="11" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G24" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H24" s="10" t="inlineStr">
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
         <is>
           <t>Completa. Tu carpeta lleva solo tu apellido, y tu respuesta sobre por que no cambio la pagina no es correcta. Ver tu hoja.</t>
         </is>
@@ -1448,22 +1445,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>tarde</t>
         </is>
       </c>
-      <c r="F25" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G25" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H25" s="10" t="inlineStr">
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1485,27 +1482,27 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>tarde</t>
         </is>
       </c>
-      <c r="F26" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H26" s="10" t="inlineStr">
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
         <is>
           <t>Completa y muy bien documentada.</t>
         </is>
@@ -1522,12 +1519,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>parcial</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1537,19 +1534,19 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H27" s="10" t="inlineStr">
-        <is>
-          <t>Falta la salida de docker ps. Ver tu hoja.</t>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>Completa. Detalles: falto pegar tu docker ps, y tu archivo se llama evindecia.md.</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1566,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1579,17 +1576,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F28" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G28" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H28" s="10" t="inlineStr">
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
         <is>
           <t>Corregida y aceptada: tu docker ps real ya quedo en tu evidencia.</t>
         </is>
@@ -1621,17 +1618,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G29" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H29" s="10" t="inlineStr">
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1653,7 +1650,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="D30" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1663,17 +1660,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F30" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G30" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H30" s="10" t="inlineStr">
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
         <is>
           <t>Completa, y tu lectura si quedo registrada en tiempo. A tu evidencia le falta un encabezado con tu nombre.</t>
         </is>
@@ -1695,7 +1692,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1705,17 +1702,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G31" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H31" s="10" t="inlineStr">
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H31" s="9" t="inlineStr">
         <is>
           <t>Completa. Listaste docker system prune, que la guia pide no usar.</t>
         </is>
@@ -1737,7 +1734,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D32" s="9" t="inlineStr">
+      <c r="D32" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1747,17 +1744,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F32" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G32" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H32" s="10" t="inlineStr">
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
         <is>
           <t>Completa. Tu archivo deberia llamarse evidencia.md, sin espacios.</t>
         </is>
@@ -1779,7 +1776,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D33" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1789,17 +1786,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F33" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G33" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H33" s="10" t="inlineStr">
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H33" s="9" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1821,7 +1818,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="D34" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1831,17 +1828,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F34" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G34" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H34" s="10" t="inlineStr">
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" s="9" t="inlineStr">
         <is>
           <t>Completa. Tu markdown quedo escapado y se ve en crudo.</t>
         </is>
@@ -1863,7 +1860,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D35" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1873,17 +1870,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G35" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H35" s="10" t="inlineStr">
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="9" t="inlineStr">
         <is>
           <t>Completa. Tu p00 ya quedo corregida. Detalle: confundiste el tag v2.</t>
         </is>
@@ -1895,37 +1892,37 @@
           <t>318026644</t>
         </is>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E36" s="11" t="inlineStr">
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G36" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H36" s="10" t="inlineStr">
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H36" s="9" t="inlineStr">
         <is>
           <t>Alta reciente. Acepta la invitacion al repositorio para poder entregar: tu rama ya esta lista.</t>
         </is>
@@ -1947,7 +1944,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr">
+      <c r="D37" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1957,17 +1954,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F37" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G37" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H37" s="10" t="inlineStr">
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" s="9" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1989,27 +1986,27 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D38" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E38" s="11" t="inlineStr">
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="F38" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G38" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H38" s="10" t="inlineStr">
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H38" s="9" t="inlineStr">
         <is>
           <t>Tu p00 quedo registrada y tu S02 ya cuenta como entregada. Te faltan las dos correcciones de tu hoja.</t>
         </is>
@@ -2041,17 +2038,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F39" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G39" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H39" s="10" t="inlineStr">
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="9" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -2068,32 +2065,32 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C40" s="8" t="inlineStr">
+      <c r="C40" s="11" t="inlineStr">
         <is>
           <t>parcial</t>
         </is>
       </c>
-      <c r="D40" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E40" s="11" t="inlineStr">
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E40" s="10" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="F40" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G40" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H40" s="10" t="inlineStr">
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H40" s="9" t="inlineStr">
         <is>
           <t>Tu docker ps no corresponde a tus contenedores y falta la tabla de comandos. Ver tu hoja.</t>
         </is>
@@ -2115,7 +2112,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D41" s="9" t="inlineStr">
+      <c r="D41" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2125,17 +2122,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F41" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G41" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H41" s="10" t="inlineStr">
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H41" s="9" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -2157,27 +2154,27 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D42" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E42" s="11" t="inlineStr">
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="F42" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G42" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H42" s="10" t="inlineStr">
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H42" s="9" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -2194,12 +2191,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C43" s="8" t="inlineStr">
+      <c r="C43" s="11" t="inlineStr">
         <is>
           <t>parcial</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr">
+      <c r="D43" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2209,17 +2206,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F43" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G43" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H43" s="10" t="inlineStr">
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H43" s="9" t="inlineStr">
         <is>
           <t>Tu evidencia quedo cortada a la mitad. Ver tu hoja.</t>
         </is>
@@ -2241,7 +2238,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D44" s="9" t="inlineStr">
+      <c r="D44" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2251,17 +2248,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F44" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G44" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H44" s="10" t="inlineStr">
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H44" s="9" t="inlineStr">
         <is>
           <t>Completa. Tu evidencia tiene los acentos rotos; guardala como UTF-8.</t>
         </is>
@@ -2283,7 +2280,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D45" s="9" t="inlineStr">
+      <c r="D45" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2293,17 +2290,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F45" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G45" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H45" s="10" t="inlineStr">
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H45" s="9" t="inlineStr">
         <is>
           <t>Completa. Tu evidencia quedo dentro de un bloque de codigo sin cerrar.</t>
         </is>
@@ -2335,17 +2332,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F46" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G46" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H46" s="10" t="inlineStr">
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H46" s="9" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -2367,7 +2364,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D47" s="9" t="inlineStr">
+      <c r="D47" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2377,17 +2374,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F47" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G47" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H47" s="10" t="inlineStr">
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" s="9" t="inlineStr">
         <is>
           <t>Completa. Tu docker ps esta recortado; pegalo completo.</t>
         </is>
@@ -2419,17 +2416,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F48" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G48" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H48" s="10" t="inlineStr">
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="inlineStr">
         <is>
           <t>Completa. Una linea de comandos quedo corrupta al pegar.</t>
         </is>
@@ -2451,7 +2448,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D49" s="9" t="inlineStr">
+      <c r="D49" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2466,12 +2463,12 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G49" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H49" s="10" t="inlineStr">
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H49" s="9" t="inlineStr">
         <is>
           <t>Completa. Usaste tags propios en vez de mi-sitio.</t>
         </is>
@@ -2493,7 +2490,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="D50" s="9" t="inlineStr">
+      <c r="D50" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -2503,17 +2500,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F50" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G50" s="9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H50" s="10" t="inlineStr">
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H50" s="9" t="inlineStr">
         <is>
           <t>Completa y correcta, y tu lectura entro en tiempo.</t>
         </is>
@@ -2536,7 +2533,7 @@
     <row r="54">
       <c r="A54" s="14" t="inlineStr">
         <is>
-          <t>S02 completa: 34 / 43   ·   parcial: 5   ·   sin entregar: 4</t>
+          <t>S02 completa: 37 / 43   ·   parcial: 2   ·   sin entregar: 4</t>
         </is>
       </c>
     </row>
@@ -2564,7 +2561,7 @@
     <row r="58">
       <c r="A58" s="14" t="inlineStr">
         <is>
-          <t>Tarea opcional (idempotency key): 0 / 43 — sigue abierta, no afecta la calificacion</t>
+          <t>Idempotency key (tarea extra): 0 / 43 — sigue abierta, es opcional y no afecta la calificacion</t>
         </is>
       </c>
     </row>
@@ -2574,149 +2571,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>Correccion · 320229264</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 320229264   ·   Por corregir: S02</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: ✓      S02: parcial      L2: ✗</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>El docker ps que pegaste no muestra tus contenedores: salen miweb, web1 y web2, no los tuyos. La mision 3 se queda sin evidencia.</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Levanta TUS dos contenedores con --name sitio y --name sitio2, corre docker ps y pega esa salida.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>El error de puerto lo describes con tus palabras ('Docker mostro un error equivalente al siguiente') en vez de pegarlo.</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Reproducelo y pega el texto tal cual sale en tu terminal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
-        <is>
-          <t>Tu index.html no trae la tabla de 5 comandos.</t>
-        </is>
-      </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>Esa era la mision 1: agregala.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="19" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="20" t="inlineStr">
-        <is>
-          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2732,244 +2586,6 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 320284858</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 320284858   ·   Por corregir: p00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: ✓      S02: ✓      L2: ✗</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Tu p00 dice solo 'prueba', sin tu nombre.</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Abrelo, escribe tu nombre completo y haz push. Tu S02 esta completa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>Correccion · 320224159</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 320224159   ·   Por corregir: S02</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: ✓      S02: parcial      L2: ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Tu evidencia.md esta cortada a la mitad: son 516 caracteres y termina a media instruccion, despues de la lista de comandos.</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Falta el docker ps, el error de puerto ocupado y las dos respuestas. Probablemente no guardaste antes de subir: completala y vuelve a hacer push.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
           <t>Correccion · 320049376</t>
         </is>
       </c>
@@ -3079,7 +2695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -3089,21 +2705,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 423054589</t>
+          <t>Correccion · 321132477</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 423054589   ·   Por corregir: S02</t>
+          <t>Cuenta: 321132477   ·   Por corregir: S02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: parcial      L2: ✓</t>
+          <t>P00: ✓      S02: ✗      L2: tarde</t>
         </is>
       </c>
     </row>
@@ -3122,66 +2738,78 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>Tu index.html todavia dice 'Hola, soy Tu Nombre': es el texto de ejemplo de la guia, no lo cambiaste. Esa era la mision 1.</t>
+          <t>No subiste nada de la S02: falta el Dockerfile, el index.html y la evidencia.md.</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Abre tu index.html, pon tu nombre real y vuelve a construir la imagen: docker build -t mi-sitio . y levanta el contenedor otra vez.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+          <t>La guia del lab esta en labs/Lab-S02-Docker-dia-1.html. Aunque sea tarde, subela: tarde no baja puntos, pero sin entrega no hay calificacion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Tu p00 esta guardado en latin-1 y tu apellido con ñ sale roto.</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Vuelve a guardarlo eligiendo codificacion UTF-8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="19" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="19" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="19" t="inlineStr">
         <is>
-          <t>git commit -m "S02: correccion"</t>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="19" t="inlineStr">
         <is>
+          <t>git commit -m "S02: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
           <t>git push</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3208,21 +2836,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 321132477</t>
+          <t>Correccion · 320298835</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 321132477   ·   Por corregir: S02</t>
+          <t>Cuenta: 320298835   ·   Por corregir: p00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: ✗      L2: tarde</t>
+          <t>P00: ✓      S02: ✓      L2: ✓</t>
         </is>
       </c>
     </row>
@@ -3241,24 +2869,24 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>No subiste nada de la S02: falta el Dockerfile, el index.html y la evidencia.md.</t>
+          <t>Tu p00 no lleva tu nombre: dice 'esta es una prueba de git'.</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>La guia del lab esta en labs/Lab-S02-Docker-dia-1.html. Aunque sea tarde, subela: tarde no baja puntos, pero sin entrega no hay calificacion.</t>
+          <t>Abrelo, escribe tu nombre completo y haz push.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>Tu p00 esta guardado en latin-1 y tu apellido con ñ sale roto.</t>
+          <t>En tu evidencia escribes docker build -t mi-sitio sin el punto final.</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Vuelve a guardarlo eligiendo codificacion UTF-8.</t>
+          <t>El punto es obligatorio: le dice a Docker donde buscar el Dockerfile.</t>
         </is>
       </c>
     </row>
@@ -3339,21 +2967,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 320298835</t>
+          <t>Correccion · 320152841</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 320298835   ·   Por corregir: p00</t>
+          <t>Cuenta: 320152841   ·   Por corregir: S02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: ✓      L2: ✓</t>
+          <t>P00: ✓      S02: ✓      L2: ✗</t>
         </is>
       </c>
     </row>
@@ -3372,24 +3000,24 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>Tu p00 no lleva tu nombre: dice 'esta es una prueba de git'.</t>
+          <t>Tu respuesta de por que la pagina no cambio esta equivocada: dices que Docker bloquea la imagen.</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Abrelo, escribe tu nombre completo y haz push.</t>
+          <t>La razon es que la imagen es inmutable: el contenedor sigue corriendo la imagen vieja, y hasta que no reconstruyes con docker build no existe una imagen nueva.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>En tu evidencia escribes docker build -t mi-sitio sin el punto final.</t>
+          <t>Tu carpeta lleva solo tu apellido.</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>El punto es obligatorio: le dice a Docker donde buscar el Dockerfile.</t>
+          <t>Deberia ser apellido_nombre, igual que tu rama.</t>
         </is>
       </c>
     </row>
@@ -3470,21 +3098,21 @@
     <row r="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
-          <t>Correccion · 117003136</t>
+          <t>Correccion · 320250648</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 117003136   ·   Por corregir: S02</t>
+          <t>Cuenta: 320250648   ·   Por corregir: p00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: ✓      S02: parcial      L2: tarde</t>
+          <t>P00: ✓      S02: ✓      L2: ✓</t>
         </is>
       </c>
     </row>
@@ -3500,27 +3128,27 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="56" customHeight="1">
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>El error que pegaste no es el que pedia la mision: pegaste 'Conflict. The container name /sitio is already in use', que es de nombre repetido. El que se pedia es el de PUERTO ocupado.</t>
+          <t>Tu p00 no lleva tu nombre.</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>Levanta dos contenedores en el MISMO puerto: docker run -d -p 9090:80 --name a mi-sitio y luego docker run -d -p 9090:80 --name b mi-sitio. El segundo falla con 'port is already allocated': pega ese texto.</t>
+          <t>Abrelo, escribe tu nombre completo y haz push.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>Tu archivo se llama Evidencia.md con mayuscula.</t>
+          <t>Tu carpeta se llama Salgado_Roman con mayusculas.</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Renombralo a evidencia.md, todo en minusculas.</t>
+          <t>Deberia ir en minusculas: apellido_nombre.</t>
         </is>
       </c>
     </row>
@@ -3586,399 +3214,6 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>Correccion · 320152841</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 320152841   ·   Por corregir: S02</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: ✓      S02: ✓      L2: ✗</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Tu respuesta de por que la pagina no cambio esta equivocada: dices que Docker bloquea la imagen.</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>La razon es que la imagen es inmutable: el contenedor sigue corriendo la imagen vieja, y hasta que no reconstruyes con docker build no existe una imagen nueva.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>Tu carpeta lleva solo tu apellido.</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Deberia ser apellido_nombre, igual que tu rama.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>Correccion · 318586465</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 318586465   ·   Por corregir: S02</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: ✓      S02: parcial      L2: ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Falta la salida de docker ps (mision 3): no aparece en tu evidencia.</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Con tus dos contenedores corriendo, ejecuta docker ps y pega la salida COMPLETA en tu evidencia.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>Tu archivo se llama evindecia.md.</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Renombralo a evidencia.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>Correccion · 320250648</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 320250648   ·   Por corregir: p00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: ✓      S02: ✓      L2: ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>Tu p00 no lleva tu nombre.</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t>Abrelo, escribe tu nombre completo y haz push.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>Tu carpeta se llama Salgado_Roman con mayusculas.</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Deberia ir en minusculas: apellido_nombre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/sNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
-        <is>
-          <t>git commit -m "S02: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4119,4 +3354,385 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Correccion · 320229264</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 320229264   ·   Por corregir: S02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>P00: ✓      S02: parcial      L2: ✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>El docker ps que pegaste no muestra tus contenedores: salen miweb, web1 y web2, no los tuyos. La mision 3 se queda sin evidencia.</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Levanta TUS dos contenedores con --name sitio y --name sitio2, corre docker ps y pega esa salida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>El error de puerto lo describes con tus palabras ('Docker mostro un error equivalente al siguiente') en vez de pegarlo.</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Reproducelo y pega el texto tal cual sale en tu terminal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Tu index.html no trae la tabla de 5 comandos.</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Esa era la mision 1: agregala.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>git commit -m "S02: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Correccion · 320284858</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 320284858   ·   Por corregir: p00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>P00: ✓      S02: ✓      L2: ✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Tu p00 dice solo 'prueba', sin tu nombre.</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Abrelo, escribe tu nombre completo y haz push. Tu S02 esta completa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>git commit -m "S02: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Correccion · 320224159</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 320224159   ·   Por corregir: S02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>P00: ✓      S02: parcial      L2: ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>Tu evidencia.md esta cortada a la mitad: son 516 caracteres y termina a media instruccion, despues de la lista de comandos.</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Falta el docker ps, el error de puerto ocupado y las dos respuestas. Probablemente no guardaste antes de subir: completala y vuelve a hacer push.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/sNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>git commit -m "S02: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Corte SD al 12-sep: incluye la S04 y la lectura 3 cerrada
</commit_message>
<xml_diff>
--- a/calificaciones/P00-S02-corte-07sep.xlsx
+++ b/calificaciones/P00-S02-corte-07sep.xlsx
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,6 +80,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00166534"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00991B1B"/>
       <sz val="10"/>
     </font>
@@ -124,7 +130,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -134,6 +140,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
     <fill>
@@ -178,7 +189,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -196,30 +207,33 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -585,17 +599,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="66" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -622,7 +637,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>L1 era opcional. L2 cerro el sabado 06-sep 06:59 (tarde: hasta el domingo). L3 sigue abierta hasta el sabado 13-sep 06:59. Idempotency key = la tarea EXTRA de entregas/OPCIONALES.md: es opcional, no afecta tu calificacion y cuenta para los puntos extra del final.</t>
+          <t>L1 era opcional. L2 cerro el sabado 06-sep 06:59 (tarde: hasta el domingo). L3 sigue abierta hasta el sabado 13-sep 06:59. S04 = el lab de Docker dia 2, vence el domingo 13 (aun abierto; aqui solo se marca si ya esta subido, el contenido se revisa al cierre). Idempotency key = la tarea EXTRA de entregas/OPCIONALES.md: es opcional, no afecta tu calificacion y cuenta para los puntos extra del final.</t>
         </is>
       </c>
     </row>
@@ -659,10 +674,15 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
+          <t>S04</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
           <t>Idempotency key</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -694,17 +714,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
         <is>
           <t>Completa. Detalle: tu index.html se quedo con el nombre de ejemplo de la guia.</t>
         </is>
@@ -721,7 +746,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -731,22 +756,27 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
         <is>
           <t>Ya hiciste tu primer push. Falta toda la S02.</t>
         </is>
@@ -783,12 +813,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H9" s="9" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -805,7 +840,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -815,22 +850,27 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>tarde</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H10" s="9" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
         <is>
           <t>Tus lecturas SI estan registradas. Falta la S02: cuando la subas se actualiza.</t>
         </is>
@@ -862,17 +902,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
         <is>
           <t>Completa. Detalle: en la evidencia falta el punto de contexto del build.</t>
         </is>
@@ -904,17 +949,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -926,12 +976,12 @@
           <t>320237012</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>BAJA</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>BAJA</t>
         </is>
@@ -941,7 +991,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -956,7 +1006,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr">
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
         <is>
           <t>Baja.</t>
         </is>
@@ -988,17 +1043,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G14" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H14" s="9" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
         <is>
           <t>Completa. Te quedo un hola_mundo.py suelto en la carpeta.</t>
         </is>
@@ -1030,17 +1090,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H15" s="9" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1072,17 +1137,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu S02 estaba en una rama vieja; ya la movimos a tu rama.</t>
         </is>
@@ -1109,22 +1179,27 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>tarde</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H17" s="9" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
         <is>
           <t>Completa. Detalle: el error que pegaste no es el de puerto ocupado, sino el de nombre repetido.</t>
         </is>
@@ -1156,17 +1231,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F18" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" s="9" t="inlineStr">
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu entrega estaba en tu rama vieja y no la habiamos visto: ya la consolidamos en tu rama. Tu evidencia esta muy bien. Detalle menor: en p00 te quedaron archivos de mas.</t>
         </is>
@@ -1198,17 +1278,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H19" s="9" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
         <is>
           <t>Completa y bien organizada.</t>
         </is>
@@ -1220,12 +1305,12 @@
           <t>114001456</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -1235,7 +1320,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -1245,12 +1330,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G20" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H20" s="9" t="inlineStr">
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
         <is>
           <t>Sin entregas registradas.</t>
         </is>
@@ -1277,22 +1367,27 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>tarde</t>
         </is>
       </c>
-      <c r="F21" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H21" s="9" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu docker ps esta recortado a mano; pegalo tal cual sale.</t>
         </is>
@@ -1324,17 +1419,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H22" s="9" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu S02 estaba en una rama vieja y tu carpeta tenia otro nombre; ya las acomodamos.</t>
         </is>
@@ -1371,12 +1471,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H23" s="9" t="inlineStr">
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1403,7 +1508,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E24" s="10" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -1413,12 +1518,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G24" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H24" s="9" t="inlineStr">
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu carpeta lleva solo tu apellido, y tu respuesta sobre por que no cambio la pagina no es correcta. Ver tu hoja.</t>
         </is>
@@ -1445,22 +1555,27 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>tarde</t>
         </is>
       </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H25" s="9" t="inlineStr">
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1487,22 +1602,27 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E26" s="11" t="inlineStr">
+      <c r="E26" s="12" t="inlineStr">
         <is>
           <t>tarde</t>
         </is>
       </c>
-      <c r="F26" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G26" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H26" s="9" t="inlineStr">
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
         <is>
           <t>Completa y muy bien documentada.</t>
         </is>
@@ -1534,17 +1654,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H27" s="9" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I27" s="10" t="inlineStr">
         <is>
           <t>Completa. Detalles: falto pegar tu docker ps, y tu archivo se llama evindecia.md.</t>
         </is>
@@ -1576,17 +1701,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F28" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G28" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H28" s="9" t="inlineStr">
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="inlineStr">
         <is>
           <t>Corregida y aceptada: tu docker ps real ya quedo en tu evidencia.</t>
         </is>
@@ -1618,17 +1748,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H29" s="9" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G29" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I29" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1660,17 +1795,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G30" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H30" s="9" t="inlineStr">
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I30" s="10" t="inlineStr">
         <is>
           <t>Completa, y tu lectura si quedo registrada en tiempo. A tu evidencia le falta un encabezado con tu nombre.</t>
         </is>
@@ -1702,17 +1842,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G31" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H31" s="9" t="inlineStr">
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I31" s="10" t="inlineStr">
         <is>
           <t>Completa. Listaste docker system prune, que la guia pide no usar.</t>
         </is>
@@ -1744,17 +1889,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F32" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G32" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H32" s="9" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I32" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu archivo deberia llamarse evidencia.md, sin espacios.</t>
         </is>
@@ -1786,17 +1936,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F33" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G33" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H33" s="9" t="inlineStr">
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I33" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1828,17 +1983,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F34" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G34" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H34" s="9" t="inlineStr">
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I34" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu markdown quedo escapado y se ve en crudo.</t>
         </is>
@@ -1870,17 +2030,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F35" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G35" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H35" s="9" t="inlineStr">
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I35" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu p00 ya quedo corregida. Detalle: confundiste el tag v2.</t>
         </is>
@@ -1892,12 +2057,12 @@
           <t>318026644</t>
         </is>
       </c>
-      <c r="B36" s="10" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="C36" s="10" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -1907,7 +2072,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E36" s="10" t="inlineStr">
+      <c r="E36" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -1917,12 +2082,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G36" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H36" s="9" t="inlineStr">
+      <c r="G36" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I36" s="10" t="inlineStr">
         <is>
           <t>Alta reciente. Acepta la invitacion al repositorio para poder entregar: tu rama ya esta lista.</t>
         </is>
@@ -1954,17 +2124,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F37" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G37" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H37" s="9" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G37" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I37" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -1991,7 +2166,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E38" s="10" t="inlineStr">
+      <c r="E38" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -2001,12 +2176,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G38" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H38" s="9" t="inlineStr">
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I38" s="10" t="inlineStr">
         <is>
           <t>Tu p00 quedo registrada y tu S02 ya cuenta como entregada. Te faltan las dos correcciones de tu hoja.</t>
         </is>
@@ -2038,17 +2218,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F39" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G39" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H39" s="9" t="inlineStr">
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I39" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -2065,7 +2250,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C40" s="11" t="inlineStr">
+      <c r="C40" s="12" t="inlineStr">
         <is>
           <t>parcial</t>
         </is>
@@ -2075,7 +2260,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E40" s="10" t="inlineStr">
+      <c r="E40" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -2085,12 +2270,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="G40" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H40" s="9" t="inlineStr">
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I40" s="10" t="inlineStr">
         <is>
           <t>Tu docker ps no corresponde a tus contenedores y falta la tabla de comandos. Ver tu hoja.</t>
         </is>
@@ -2122,17 +2312,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F41" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G41" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H41" s="9" t="inlineStr">
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I41" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -2159,22 +2354,27 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E42" s="10" t="inlineStr">
+      <c r="E42" s="11" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="F42" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G42" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H42" s="9" t="inlineStr">
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G42" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I42" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -2191,7 +2391,7 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="C43" s="11" t="inlineStr">
+      <c r="C43" s="12" t="inlineStr">
         <is>
           <t>parcial</t>
         </is>
@@ -2206,17 +2406,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F43" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G43" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H43" s="9" t="inlineStr">
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I43" s="10" t="inlineStr">
         <is>
           <t>Tu evidencia quedo cortada a la mitad. Ver tu hoja.</t>
         </is>
@@ -2248,17 +2453,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F44" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G44" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H44" s="9" t="inlineStr">
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I44" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu evidencia tiene los acentos rotos; guardala como UTF-8.</t>
         </is>
@@ -2290,17 +2500,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F45" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G45" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H45" s="9" t="inlineStr">
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I45" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu evidencia quedo dentro de un bloque de codigo sin cerrar.</t>
         </is>
@@ -2332,17 +2547,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F46" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G46" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H46" s="9" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I46" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta.</t>
         </is>
@@ -2374,17 +2594,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F47" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G47" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H47" s="9" t="inlineStr">
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G47" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I47" s="10" t="inlineStr">
         <is>
           <t>Completa. Tu docker ps esta recortado; pegalo completo.</t>
         </is>
@@ -2416,17 +2641,22 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F48" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G48" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H48" s="9" t="inlineStr">
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G48" s="11" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="H48" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I48" s="10" t="inlineStr">
         <is>
           <t>Completa. Una linea de comandos quedo corrupta al pegar.</t>
         </is>
@@ -2463,12 +2693,17 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="G49" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H49" s="9" t="inlineStr">
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H49" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I49" s="10" t="inlineStr">
         <is>
           <t>Completa. Usaste tags propios en vez de mi-sitio.</t>
         </is>
@@ -2500,66 +2735,78 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="F50" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G50" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H50" s="9" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>subida</t>
+        </is>
+      </c>
+      <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I50" s="10" t="inlineStr">
         <is>
           <t>Completa y correcta, y tu lectura entro en tiempo.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="13" t="inlineStr">
+      <c r="A52" s="14" t="inlineStr">
         <is>
           <t>Resumen del grupo (43 alumnos activos · 1 baja no contada)</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="14" t="inlineStr">
+      <c r="A53" s="15" t="inlineStr">
         <is>
           <t>P00 entregada: 41 / 43   (de esas, 0 sin el nombre adentro)</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="14" t="inlineStr">
+      <c r="A54" s="15" t="inlineStr">
         <is>
           <t>S02 completa: 37 / 43   ·   parcial: 2   ·   sin entregar: 4</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="14" t="inlineStr">
+      <c r="A55" s="15" t="inlineStr">
         <is>
           <t>Lectura 2: 31 en tiempo + 5 tarde = 36 / 43</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="14" t="inlineStr">
-        <is>
-          <t>Lectura 3 (abierta hasta el 13-sep): 1 / 43</t>
+      <c r="A56" s="15" t="inlineStr">
+        <is>
+          <t>Lectura 3 (cerro el 12-sep 06:59): 36 / 43 — todos en tiempo</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="14" t="inlineStr">
+      <c r="A57" s="15" t="inlineStr">
+        <is>
+          <t>Lab S04 (vence el domingo 13): 18 / 43 ya subido</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="15" t="inlineStr">
         <is>
           <t>Sin absolutamente nada: 2 / 43</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="14" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
         <is>
           <t>Idempotency key (tarea extra): 0 / 43 — sigue abierta, es opcional y no afecta la calificacion</t>
         </is>
@@ -2584,7 +2831,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Correccion · 320049376</t>
         </is>
@@ -2598,87 +2845,87 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>P00: ✓      S02: ✓      L2: ✓</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>No tienes p00, que era la primera tarea de Git.</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Crea entregas/tu_carpeta/p00/prueba.txt con tu nombre completo adentro y haz push. Tu S02 si esta completa.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2703,7 +2950,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Correccion · 321132477</t>
         </is>
@@ -2717,99 +2964,99 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>P00: ✓      S02: ✗      L2: tarde</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>No subiste nada de la S02: falta el Dockerfile, el index.html y la evidencia.md.</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>La guia del lab esta en labs/Lab-S02-Docker-dia-1.html. Aunque sea tarde, subela: tarde no baja puntos, pero sin entrega no hay calificacion.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Tu p00 esta guardado en latin-1 y tu apellido con ñ sale roto.</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Vuelve a guardarlo eligiendo codificacion UTF-8.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2834,7 +3081,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Correccion · 320298835</t>
         </is>
@@ -2848,99 +3095,99 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>P00: ✓      S02: ✓      L2: ✓</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Tu p00 no lleva tu nombre: dice 'esta es una prueba de git'.</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Abrelo, escribe tu nombre completo y haz push.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>En tu evidencia escribes docker build -t mi-sitio sin el punto final.</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>El punto es obligatorio: le dice a Docker donde buscar el Dockerfile.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2965,7 +3212,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Correccion · 320152841</t>
         </is>
@@ -2979,99 +3226,99 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>P00: ✓      S02: ✓      L2: ✗</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Tu respuesta de por que la pagina no cambio esta equivocada: dices que Docker bloquea la imagen.</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>La razon es que la imagen es inmutable: el contenedor sigue corriendo la imagen vieja, y hasta que no reconstruyes con docker build no existe una imagen nueva.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Tu carpeta lleva solo tu apellido.</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Deberia ser apellido_nombre, igual que tu rama.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3096,7 +3343,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Correccion · 320250648</t>
         </is>
@@ -3110,99 +3357,99 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>P00: ✓      S02: ✓      L2: ✓</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Tu p00 no lleva tu nombre.</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Abrelo, escribe tu nombre completo y haz push.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Tu carpeta se llama Salgado_Roman con mayusculas.</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Deberia ir en minusculas: apellido_nombre.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3227,7 +3474,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Correccion · 319659852</t>
         </is>
@@ -3241,111 +3488,111 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>P00: ✓      S02: ✓      L2: ✗</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Falta el error de puerto ocupado: no aparece en tu evidencia.</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Levanta dos contenedores en el mismo puerto; el segundo falla con 'port is already allocated'. Pega ese texto en tu evidencia.md.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Tu Dockerfile es el unico sin EXPOSE 80.</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Agregale la linea EXPOSE 80 . Construye igual, pero documenta que el contenedor escucha en ese puerto.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Tu p00 ya quedo registrada, esa ya no le muevas.</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Tu S02 ya cuenta como entregada: estas dos correcciones son para dejarla completa.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3370,7 +3617,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Correccion · 320229264</t>
         </is>
@@ -3384,111 +3631,111 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>P00: ✓      S02: parcial      L2: ✗</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>El docker ps que pegaste no muestra tus contenedores: salen miweb, web1 y web2, no los tuyos. La mision 3 se queda sin evidencia.</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Levanta TUS dos contenedores con --name sitio y --name sitio2, corre docker ps y pega esa salida.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>El error de puerto lo describes con tus palabras ('Docker mostro un error equivalente al siguiente') en vez de pegarlo.</t>
         </is>
       </c>
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Reproducelo y pega el texto tal cual sale en tu terminal.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Tu index.html no trae la tabla de 5 comandos.</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Esa era la mision 1: agregala.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3513,7 +3760,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Correccion · 320284858</t>
         </is>
@@ -3527,87 +3774,87 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>P00: ✓      S02: ✓      L2: ✗</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Tu p00 dice solo 'prueba', sin tu nombre.</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Abrelo, escribe tu nombre completo y haz push. Tu S02 esta completa.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>
@@ -3632,7 +3879,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Correccion · 320224159</t>
         </is>
@@ -3646,87 +3893,87 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>P00: ✓      S02: parcial      L2: ✓</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Tu evidencia.md esta cortada a la mitad: son 516 caracteres y termina a media instruccion, despues de la lista de comandos.</t>
         </is>
       </c>
-      <c r="B6" s="17" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Falta el docker ps, el error de puerto ocupado y las dos respuestas. Probablemente no guardaste antes de subir: completala y vuelve a hacer push.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/sNN</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>git commit -m "S02: correccion"</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>Entregar tarde no baja puntos, pero se registra. No abras pull request: el push ES la entrega.</t>
         </is>

</xml_diff>